<commit_message>
updated feature - added new look -searchable -dark mode -tab page name updated - autofetch icons
</commit_message>
<xml_diff>
--- a/bookmarks.xlsx
+++ b/bookmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gitvolume\html_bookmarks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD123B0-2E79-4225-8012-73A32C3812A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9276F9-E3DD-4184-853E-680482030349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="12" r:id="rId1"/>
@@ -1261,9 +1261,6 @@
     <t>LTTS HOME</t>
   </si>
   <si>
-    <t>https://myts.ltts.com/Home</t>
-  </si>
-  <si>
     <t>LTTS</t>
   </si>
   <si>
@@ -1301,6 +1298,9 @@
   </si>
   <si>
     <t>https://static1.anpoimages.com/wordpress/wp-content/uploads/2023/10/how-to-create-a-gantt-chart-in-google-sheets-logo.jpg</t>
+  </si>
+  <si>
+    <t>https://myltts.ltts.com/home</t>
   </si>
 </sst>
 </file>
@@ -1433,38 +1433,30 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
+  <dxfs count="16">
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC65911"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF548235"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -1497,102 +1489,6 @@
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC65911"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF548235"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC65911"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF548235"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC65911"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF548235"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1653,19 +1549,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{03E3FB43-9AEF-40D1-8FBE-6434E6283EA1}" name="Table3" displayName="Table3" ref="A1:D140" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{03E3FB43-9AEF-40D1-8FBE-6434E6283EA1}" name="Table3" displayName="Table3" ref="A1:D140" headerRowDxfId="15" dataDxfId="13" headerRowBorderDxfId="14" tableBorderDxfId="12">
   <autoFilter ref="A1:D140" xr:uid="{03E3FB43-9AEF-40D1-8FBE-6434E6283EA1}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D140">
-    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="7"/>
-    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="6"/>
-    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="5"/>
-    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="4"/>
+    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="11"/>
+    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="10"/>
+    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="9"/>
+    <sortCondition sortBy="cellColor" ref="C2:C140" dxfId="8"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{FF371AF1-99C5-4AAC-BB80-035E3D76979B}" name="title" totalsRowLabel="Total" dataDxfId="24" totalsRowDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{3693D4F3-FFA3-4FC1-92A0-DB464B710988}" name="url" dataDxfId="22" totalsRowDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{D68EC384-C9FA-42C9-A1F7-3B3C2801C07F}" name="category" dataDxfId="20" totalsRowDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{6169A379-D1C5-4FFB-86EC-6185B276DF18}" name="image" totalsRowFunction="count" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{FF371AF1-99C5-4AAC-BB80-035E3D76979B}" name="title" totalsRowLabel="Total" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{3693D4F3-FFA3-4FC1-92A0-DB464B710988}" name="url" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{D68EC384-C9FA-42C9-A1F7-3B3C2801C07F}" name="category" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{6169A379-D1C5-4FFB-86EC-6185B276DF18}" name="image" totalsRowFunction="count" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2414,7 +2310,7 @@
         <v>6</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -2428,7 +2324,7 @@
         <v>6</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -2442,7 +2338,7 @@
         <v>6</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
@@ -2456,7 +2352,7 @@
         <v>6</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -2696,30 +2592,30 @@
     </row>
     <row r="55" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B56" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D56" s="1" t="s">
         <v>404</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -3790,42 +3686,42 @@
       <c r="A133" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="B133" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C133" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="C133" s="1" t="s">
-        <v>396</v>
-      </c>
       <c r="D133" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="B135" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="B135" s="1" t="s">
+      <c r="C135" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="D135" s="1" t="s">
         <v>400</v>
-      </c>
-      <c r="C135" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="D135" s="1" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
@@ -3903,10 +3799,11 @@
     <hyperlink ref="B57" r:id="rId1" xr:uid="{AA559BEB-464C-4ED1-95E5-59EDFA000179}"/>
     <hyperlink ref="D69" r:id="rId2" xr:uid="{63D81A31-8F44-45D4-A777-45B5373AABF8}"/>
     <hyperlink ref="B69" r:id="rId3" xr:uid="{60680A10-1FFE-4959-B2F7-366C1B00A63D}"/>
+    <hyperlink ref="B133" r:id="rId4" xr:uid="{C95626FA-14A8-4604-BFD5-EED429938D23}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>